<commit_message>
docs(payroll): keep summary title readable
</commit_message>
<xml_diff>
--- a/World_Concern_Financial_Workbook_for_review.xlsx
+++ b/World_Concern_Financial_Workbook_for_review.xlsx
@@ -60,7 +60,7 @@
     <col min="3" max="3" width="68" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">WORLD CONCERN PAYROLL — FINANCIAL WORKBOOK</t>
@@ -247,10 +247,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>